<commit_message>
large DCDCv9-3r1.4 release update
- Removed some tables in csv and ods format (xlsx preferred)
- fixed issue #10 (waiting for approval)
- added video of adhesive testing for ESG10C-20G
- added video of primary and secondary winding
- updated all documentation files incl. Scrutineering Support Presentation
- updated transformer isolator part
- updated build notes
- updated README.md
- updated HV input connector
- added note about the discontinuation of the German versions
- added R75 onto the PCB (not required to solder on top of R31 anymore)
- updated iBoms and comments
- removed solder mask between TS an LV for better inspection
- replaced J1, unified crimps for all molex housings
- replaced U1
- fresh production files and gerber PDF plots
</commit_message>
<xml_diff>
--- a/kicad/production/DCDCv9-3_Mouser_BOM_for_PCBA.xlsx
+++ b/kicad/production/DCDCv9-3_Mouser_BOM_for_PCBA.xlsx
@@ -11,7 +11,7 @@
     <sheet name="DCDCv9-3_kicad_full_bom" sheetId="1" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">'DCDCv9-3_kicad_full_bom'!$A$1:$L$47</definedName>
+    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">'DCDCv9-3_kicad_full_bom'!$A$1:$L$46</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
   <extLst>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="324" uniqueCount="235">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="316" uniqueCount="229">
   <si>
     <t xml:space="preserve">Reference</t>
   </si>
@@ -268,13 +268,13 @@
     <t xml:space="preserve">J1</t>
   </si>
   <si>
-    <t xml:space="preserve">Screw_Terminal_01x03</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.mouser.de/ProductDetail/TE-Connectivity/282828-2?qs=%2FmCiCROZvxYuPZyQ6f5T0w%3D%3D</t>
-  </si>
-  <si>
-    <t xml:space="preserve">282828-2</t>
+    <t xml:space="preserve">Terminal_01x03</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.mouser.de/ProductDetail/Molex/43650-0315?qs=Nb99Pa9xYq%2FPpvf19i2uYA%3D%3D</t>
+  </si>
+  <si>
+    <t xml:space="preserve">43650-0315</t>
   </si>
   <si>
     <t xml:space="preserve">DCDC-Footprints:TerminalBlock_TE-282817-2_1x03_P5.00mm_90 Degrees updated v9-3</t>
@@ -286,28 +286,28 @@
     <t xml:space="preserve">J1.1</t>
   </si>
   <si>
-    <t xml:space="preserve">https://www.mouser.de/ProductDetail/TE-Connectivity/284051-2?qs=OYEvAappxlxBiuwfKz%2FgFA%3D%3D</t>
-  </si>
-  <si>
-    <t xml:space="preserve">284051-2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HV Plug angled</t>
-  </si>
-  <si>
-    <t xml:space="preserve">use J1.1 or J1.2 (order both just in case)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">J1.2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.mouser.de/ProductDetail/TE-Connectivity/282809-2?qs=tAlKl34sQZui56eeBzZTxA%3D%3D</t>
-  </si>
-  <si>
-    <t xml:space="preserve">282809-2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HV Plug straight</t>
+    <t xml:space="preserve">https://www.mouser.de/ProductDetail/Molex/43645-0300?qs=W6FIH8d5%2F%2F06ciSdVM35nA%3D%3D</t>
+  </si>
+  <si>
+    <t xml:space="preserve">43645-0300</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Receptacle Housing</t>
+  </si>
+  <si>
+    <t xml:space="preserve">J1.2,J1.3,J1.4,J3.2,J3.3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Conn_01x01_Pin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.mouser.de/ProductDetail/Molex/35044-9102?qs=ZlMU7IUseCu3dWv7JcWPgw%3D%3D</t>
+  </si>
+  <si>
+    <t xml:space="preserve">35044-9102</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Crimp for molex micofit receptacle housing</t>
   </si>
   <si>
     <t xml:space="preserve">J2,J4,J8</t>
@@ -350,24 +350,6 @@
   </si>
   <si>
     <t xml:space="preserve">43645-0200</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Receptacle Housing</t>
-  </si>
-  <si>
-    <t xml:space="preserve">J3.2,J3.3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Conn_01x01_Pin</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.mouser.de/ProductDetail/Molex/35044-9102?qs=ZlMU7IUseCu3dWv7JcWPgw%3D%3D</t>
-  </si>
-  <si>
-    <t xml:space="preserve">35044-9102</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Crimp for molex micofit receptacle housing</t>
   </si>
   <si>
     <t xml:space="preserve">J5</t>
@@ -802,7 +784,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -813,6 +795,10 @@
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -951,7 +937,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:L47"/>
+  <dimension ref="A1:L46"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="61.95"/>
@@ -1360,19 +1346,19 @@
       </c>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="1" t="s">
+      <c r="A15" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="B15" s="1" t="s">
+      <c r="B15" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="C15" s="1" t="s">
+      <c r="C15" s="0" t="s">
         <v>82</v>
       </c>
-      <c r="D15" s="1" t="s">
+      <c r="D15" s="3" t="s">
         <v>83</v>
       </c>
-      <c r="E15" s="1" t="s">
+      <c r="E15" s="2" t="s">
         <v>84</v>
       </c>
       <c r="F15" s="1" t="n">
@@ -1381,51 +1367,46 @@
       <c r="H15" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="K15" s="1" t="s">
+      <c r="K15" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="L15" s="1" t="s">
+      <c r="L15" s="2" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="1" t="s">
+      <c r="A16" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="B16" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="C16" s="1" t="s">
+      <c r="B16" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="C16" s="0" t="s">
         <v>87</v>
       </c>
-      <c r="D16" s="1" t="s">
+      <c r="D16" s="3" t="s">
         <v>88</v>
       </c>
-      <c r="E16" s="1" t="s">
+      <c r="E16" s="2" t="s">
         <v>66</v>
       </c>
       <c r="F16" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="H16" s="1" t="n">
         <v>1</v>
       </c>
       <c r="J16" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="K16" s="1" t="s">
-        <v>90</v>
-      </c>
-      <c r="L16" s="1" t="s">
+      <c r="K16" s="2"/>
+      <c r="L16" s="2" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="B17" s="1" t="s">
         <v>91</v>
-      </c>
-      <c r="B17" s="1" t="s">
-        <v>81</v>
       </c>
       <c r="C17" s="1" t="s">
         <v>92</v>
@@ -1437,18 +1418,12 @@
         <v>66</v>
       </c>
       <c r="F17" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="H17" s="1" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="J17" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="K17" s="1" t="s">
-        <v>90</v>
-      </c>
-      <c r="L17" s="1" t="s">
+      <c r="L17" s="2" t="s">
         <v>17</v>
       </c>
     </row>
@@ -1527,10 +1502,10 @@
         <v>1</v>
       </c>
       <c r="J20" s="1" t="s">
-        <v>109</v>
+        <v>89</v>
       </c>
       <c r="K20" s="1" t="s">
-        <v>109</v>
+        <v>89</v>
       </c>
       <c r="L20" s="1" t="s">
         <v>17</v>
@@ -1538,24 +1513,30 @@
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="B21" s="1" t="s">
         <v>110</v>
       </c>
-      <c r="B21" s="1" t="s">
+      <c r="C21" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="C21" s="1" t="s">
+      <c r="D21" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="E21" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="D21" s="1" t="s">
+      <c r="F21" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="H21" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="K21" s="1" t="s">
         <v>113</v>
       </c>
-      <c r="E21" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="F21" s="1" t="n">
-        <v>2</v>
-      </c>
-      <c r="J21" s="1" t="s">
+      <c r="L21" s="1" t="s">
         <v>114</v>
       </c>
     </row>
@@ -1567,106 +1548,106 @@
         <v>116</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>117</v>
+        <v>111</v>
       </c>
       <c r="D22" s="1" t="s">
         <v>66</v>
       </c>
       <c r="E22" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="F22" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="H22" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="J22" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="K22" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="F22" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="H22" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="K22" s="1" t="s">
-        <v>119</v>
-      </c>
       <c r="L22" s="1" t="s">
-        <v>120</v>
+        <v>114</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="1" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>122</v>
+        <v>96</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>117</v>
+        <v>97</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>66</v>
+        <v>98</v>
       </c>
       <c r="E23" s="1" t="s">
-        <v>66</v>
+        <v>99</v>
       </c>
       <c r="F23" s="1" t="n">
-        <v>1</v>
+        <v>2</v>
+      </c>
+      <c r="G23" s="1" t="s">
+        <v>6</v>
       </c>
       <c r="H23" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="J23" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="K23" s="1" t="s">
-        <v>124</v>
+      <c r="I23" s="1" t="n">
+        <v>1</v>
       </c>
       <c r="L23" s="1" t="s">
-        <v>120</v>
+        <v>17</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="1" t="s">
-        <v>125</v>
+        <v>120</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>96</v>
+        <v>121</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>97</v>
+        <v>66</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>98</v>
+        <v>66</v>
       </c>
       <c r="E24" s="1" t="s">
-        <v>99</v>
+        <v>122</v>
       </c>
       <c r="F24" s="1" t="n">
-        <v>2</v>
-      </c>
-      <c r="G24" s="1" t="s">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="H24" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="I24" s="1" t="n">
-        <v>1</v>
+      <c r="K24" s="1" t="s">
+        <v>123</v>
       </c>
       <c r="L24" s="1" t="s">
-        <v>17</v>
+        <v>124</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="B25" s="1" t="s">
         <v>126</v>
       </c>
-      <c r="B25" s="1" t="s">
+      <c r="C25" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="C25" s="1" t="s">
-        <v>66</v>
-      </c>
       <c r="D25" s="1" t="s">
-        <v>66</v>
+        <v>128</v>
       </c>
       <c r="E25" s="1" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="F25" s="1" t="n">
         <v>1</v>
@@ -1674,11 +1655,11 @@
       <c r="H25" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="K25" s="1" t="s">
-        <v>129</v>
+      <c r="J25" s="1" t="s">
+        <v>130</v>
       </c>
       <c r="L25" s="1" t="s">
-        <v>130</v>
+        <v>17</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1691,20 +1672,17 @@
       <c r="C26" s="1" t="s">
         <v>133</v>
       </c>
-      <c r="D26" s="1" t="s">
+      <c r="D26" s="1" t="n">
+        <v>7443091100</v>
+      </c>
+      <c r="E26" s="1" t="s">
         <v>134</v>
       </c>
-      <c r="E26" s="1" t="s">
-        <v>135</v>
-      </c>
       <c r="F26" s="1" t="n">
         <v>1</v>
       </c>
       <c r="H26" s="1" t="n">
         <v>1</v>
-      </c>
-      <c r="J26" s="1" t="s">
-        <v>136</v>
       </c>
       <c r="L26" s="1" t="s">
         <v>17</v>
@@ -1712,25 +1690,28 @@
     </row>
     <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="B27" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="C27" s="1" t="s">
         <v>137</v>
       </c>
-      <c r="B27" s="1" t="s">
+      <c r="D27" s="1" t="s">
         <v>138</v>
       </c>
-      <c r="C27" s="1" t="s">
+      <c r="E27" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="F27" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="H27" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="J27" s="1" t="s">
         <v>139</v>
-      </c>
-      <c r="D27" s="1" t="n">
-        <v>7443091100</v>
-      </c>
-      <c r="E27" s="1" t="s">
-        <v>140</v>
-      </c>
-      <c r="F27" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="H27" s="1" t="n">
-        <v>1</v>
       </c>
       <c r="L27" s="1" t="s">
         <v>17</v>
@@ -1738,77 +1719,74 @@
     </row>
     <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="B28" s="1" t="s">
         <v>141</v>
       </c>
-      <c r="B28" s="1" t="s">
+      <c r="C28" s="1" t="s">
         <v>142</v>
       </c>
-      <c r="C28" s="1" t="s">
-        <v>143</v>
-      </c>
       <c r="D28" s="1" t="s">
-        <v>144</v>
+        <v>66</v>
       </c>
       <c r="E28" s="1" t="s">
-        <v>135</v>
+        <v>99</v>
       </c>
       <c r="F28" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="H28" s="1" t="n">
-        <v>1</v>
-      </c>
       <c r="J28" s="1" t="s">
-        <v>145</v>
+        <v>141</v>
       </c>
       <c r="L28" s="1" t="s">
-        <v>17</v>
+        <v>114</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="B29" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="C29" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="D29" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="E29" s="1" t="s">
         <v>146</v>
       </c>
-      <c r="B29" s="1" t="s">
-        <v>147</v>
-      </c>
-      <c r="C29" s="1" t="s">
-        <v>148</v>
-      </c>
-      <c r="D29" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="E29" s="1" t="s">
-        <v>99</v>
-      </c>
       <c r="F29" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="J29" s="1" t="s">
-        <v>147</v>
+        <v>2</v>
+      </c>
+      <c r="H29" s="1" t="n">
+        <v>1</v>
       </c>
       <c r="L29" s="1" t="s">
-        <v>120</v>
+        <v>17</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="1" t="s">
+        <v>147</v>
+      </c>
+      <c r="B30" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="C30" s="1" t="s">
         <v>149</v>
       </c>
-      <c r="B30" s="1" t="s">
+      <c r="D30" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="E30" s="1" t="s">
         <v>150</v>
       </c>
-      <c r="C30" s="1" t="s">
-        <v>151</v>
-      </c>
-      <c r="D30" s="1" t="s">
-        <v>150</v>
-      </c>
-      <c r="E30" s="1" t="s">
-        <v>152</v>
-      </c>
       <c r="F30" s="1" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H30" s="1" t="n">
         <v>1</v>
@@ -1819,19 +1797,19 @@
     </row>
     <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="1" t="s">
+        <v>151</v>
+      </c>
+      <c r="B31" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="C31" s="1" t="s">
         <v>153</v>
       </c>
-      <c r="B31" s="1" t="s">
-        <v>154</v>
-      </c>
-      <c r="C31" s="1" t="s">
-        <v>155</v>
-      </c>
       <c r="D31" s="1" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="E31" s="1" t="s">
-        <v>156</v>
+        <v>150</v>
       </c>
       <c r="F31" s="1" t="n">
         <v>1</v>
@@ -1845,25 +1823,28 @@
     </row>
     <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="B32" s="1" t="s">
+        <v>155</v>
+      </c>
+      <c r="C32" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="D32" s="1" t="s">
         <v>157</v>
       </c>
-      <c r="B32" s="1" t="s">
+      <c r="E32" s="1" t="s">
         <v>158</v>
       </c>
-      <c r="C32" s="1" t="s">
+      <c r="F32" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="I32" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="K32" s="1" t="s">
         <v>159</v>
-      </c>
-      <c r="D32" s="1" t="s">
-        <v>158</v>
-      </c>
-      <c r="E32" s="1" t="s">
-        <v>156</v>
-      </c>
-      <c r="F32" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="H32" s="1" t="n">
-        <v>1</v>
       </c>
       <c r="L32" s="1" t="s">
         <v>17</v>
@@ -1917,7 +1898,7 @@
       <c r="F34" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="I34" s="1" t="n">
+      <c r="H34" s="1" t="n">
         <v>1</v>
       </c>
       <c r="K34" s="1" t="s">
@@ -1938,19 +1919,22 @@
         <v>174</v>
       </c>
       <c r="D35" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="E35" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="F35" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="H35" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="J35" s="1" t="s">
         <v>175</v>
       </c>
-      <c r="E35" s="1" t="s">
-        <v>176</v>
-      </c>
-      <c r="F35" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="H35" s="1" t="n">
-        <v>1</v>
-      </c>
       <c r="K35" s="1" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="L35" s="1" t="s">
         <v>17</v>
@@ -1958,16 +1942,16 @@
     </row>
     <row r="36" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="1" t="s">
+        <v>176</v>
+      </c>
+      <c r="B36" s="1" t="s">
+        <v>177</v>
+      </c>
+      <c r="C36" s="1" t="s">
         <v>178</v>
       </c>
-      <c r="B36" s="1" t="s">
+      <c r="D36" s="1" t="s">
         <v>179</v>
-      </c>
-      <c r="C36" s="1" t="s">
-        <v>180</v>
-      </c>
-      <c r="D36" s="1" t="s">
-        <v>175</v>
       </c>
       <c r="E36" s="1" t="s">
         <v>66</v>
@@ -1979,10 +1963,10 @@
         <v>1</v>
       </c>
       <c r="J36" s="1" t="s">
-        <v>181</v>
+        <v>175</v>
       </c>
       <c r="K36" s="1" t="s">
-        <v>181</v>
+        <v>175</v>
       </c>
       <c r="L36" s="1" t="s">
         <v>17</v>
@@ -1990,16 +1974,16 @@
     </row>
     <row r="37" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="1" t="s">
+        <v>180</v>
+      </c>
+      <c r="B37" s="1" t="s">
+        <v>181</v>
+      </c>
+      <c r="C37" s="1" t="s">
         <v>182</v>
       </c>
-      <c r="B37" s="1" t="s">
+      <c r="D37" s="1" t="s">
         <v>183</v>
-      </c>
-      <c r="C37" s="1" t="s">
-        <v>184</v>
-      </c>
-      <c r="D37" s="1" t="s">
-        <v>185</v>
       </c>
       <c r="E37" s="1" t="s">
         <v>66</v>
@@ -2007,92 +1991,89 @@
       <c r="F37" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="H37" s="1" t="n">
-        <v>1</v>
-      </c>
       <c r="J37" s="1" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="K37" s="1" t="s">
-        <v>181</v>
+        <v>185</v>
       </c>
       <c r="L37" s="1" t="s">
-        <v>17</v>
+        <v>186</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="1" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="C38" s="1" t="s">
-        <v>188</v>
+        <v>182</v>
       </c>
       <c r="D38" s="1" t="s">
-        <v>189</v>
+        <v>183</v>
       </c>
       <c r="E38" s="1" t="s">
         <v>66</v>
       </c>
       <c r="F38" s="1" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J38" s="1" t="s">
-        <v>190</v>
+        <v>184</v>
       </c>
       <c r="K38" s="1" t="s">
-        <v>191</v>
+        <v>185</v>
       </c>
       <c r="L38" s="1" t="s">
-        <v>192</v>
+        <v>186</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="1" t="s">
+        <v>189</v>
+      </c>
+      <c r="B39" s="1" t="s">
+        <v>190</v>
+      </c>
+      <c r="C39" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="D39" s="1" t="s">
+        <v>192</v>
+      </c>
+      <c r="E39" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="F39" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="H39" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="K39" s="1" t="s">
         <v>193</v>
       </c>
-      <c r="B39" s="1" t="s">
-        <v>194</v>
-      </c>
-      <c r="C39" s="1" t="s">
-        <v>188</v>
-      </c>
-      <c r="D39" s="1" t="s">
-        <v>189</v>
-      </c>
-      <c r="E39" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="F39" s="1" t="n">
-        <v>2</v>
-      </c>
-      <c r="J39" s="1" t="s">
-        <v>190</v>
-      </c>
-      <c r="K39" s="1" t="s">
-        <v>191</v>
-      </c>
       <c r="L39" s="1" t="s">
-        <v>192</v>
+        <v>17</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="1" t="s">
+        <v>194</v>
+      </c>
+      <c r="B40" s="1" t="s">
         <v>195</v>
       </c>
-      <c r="B40" s="1" t="s">
+      <c r="C40" s="1" t="s">
         <v>196</v>
       </c>
-      <c r="C40" s="1" t="s">
+      <c r="D40" s="1" t="s">
         <v>197</v>
       </c>
-      <c r="D40" s="1" t="s">
+      <c r="E40" s="1" t="s">
         <v>198</v>
-      </c>
-      <c r="E40" s="1" t="s">
-        <v>99</v>
       </c>
       <c r="F40" s="1" t="n">
         <v>1</v>
@@ -2118,19 +2099,19 @@
         <v>202</v>
       </c>
       <c r="D41" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="E41" s="1" t="s">
         <v>203</v>
       </c>
-      <c r="E41" s="1" t="s">
+      <c r="F41" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="H41" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="J41" s="1" t="s">
         <v>204</v>
-      </c>
-      <c r="F41" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="H41" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="K41" s="1" t="s">
-        <v>205</v>
       </c>
       <c r="L41" s="1" t="s">
         <v>17</v>
@@ -2138,16 +2119,16 @@
     </row>
     <row r="42" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="1" t="s">
+        <v>205</v>
+      </c>
+      <c r="B42" s="1" t="s">
         <v>206</v>
       </c>
-      <c r="B42" s="1" t="s">
+      <c r="C42" s="1" t="s">
         <v>207</v>
       </c>
-      <c r="C42" s="1" t="s">
+      <c r="D42" s="1" t="s">
         <v>208</v>
-      </c>
-      <c r="D42" s="1" t="s">
-        <v>207</v>
       </c>
       <c r="E42" s="1" t="s">
         <v>209</v>
@@ -2155,10 +2136,10 @@
       <c r="F42" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="H42" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="J42" s="1" t="s">
+      <c r="I42" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="K42" s="1" t="s">
         <v>210</v>
       </c>
       <c r="L42" s="1" t="s">
@@ -2176,19 +2157,19 @@
         <v>213</v>
       </c>
       <c r="D43" s="1" t="s">
+        <v>212</v>
+      </c>
+      <c r="E43" s="1" t="s">
         <v>214</v>
       </c>
-      <c r="E43" s="1" t="s">
+      <c r="F43" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="H43" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="K43" s="1" t="s">
         <v>215</v>
-      </c>
-      <c r="F43" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="I43" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="K43" s="1" t="s">
-        <v>216</v>
       </c>
       <c r="L43" s="1" t="s">
         <v>17</v>
@@ -2196,28 +2177,28 @@
     </row>
     <row r="44" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="1" t="s">
+        <v>216</v>
+      </c>
+      <c r="B44" s="1" t="s">
         <v>217</v>
       </c>
-      <c r="B44" s="1" t="s">
+      <c r="C44" s="1" t="s">
         <v>218</v>
       </c>
-      <c r="C44" s="1" t="s">
+      <c r="D44" s="1" t="s">
+        <v>217</v>
+      </c>
+      <c r="E44" s="1" t="s">
+        <v>214</v>
+      </c>
+      <c r="F44" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="H44" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="J44" s="1" t="s">
         <v>219</v>
-      </c>
-      <c r="D44" s="1" t="s">
-        <v>218</v>
-      </c>
-      <c r="E44" s="1" t="s">
-        <v>220</v>
-      </c>
-      <c r="F44" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="H44" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="K44" s="1" t="s">
-        <v>221</v>
       </c>
       <c r="L44" s="1" t="s">
         <v>17</v>
@@ -2225,28 +2206,25 @@
     </row>
     <row r="45" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="1" t="s">
+        <v>220</v>
+      </c>
+      <c r="B45" s="1" t="s">
+        <v>221</v>
+      </c>
+      <c r="C45" s="1" t="s">
         <v>222</v>
-      </c>
-      <c r="B45" s="1" t="s">
-        <v>223</v>
-      </c>
-      <c r="C45" s="1" t="s">
-        <v>224</v>
       </c>
       <c r="D45" s="1" t="s">
         <v>223</v>
       </c>
       <c r="E45" s="1" t="s">
-        <v>220</v>
+        <v>224</v>
       </c>
       <c r="F45" s="1" t="n">
         <v>1</v>
       </c>
       <c r="H45" s="1" t="n">
         <v>1</v>
-      </c>
-      <c r="J45" s="1" t="s">
-        <v>225</v>
       </c>
       <c r="L45" s="1" t="s">
         <v>17</v>
@@ -2254,22 +2232,22 @@
     </row>
     <row r="46" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="1" t="s">
+        <v>225</v>
+      </c>
+      <c r="B46" s="1" t="s">
         <v>226</v>
       </c>
-      <c r="B46" s="1" t="s">
+      <c r="C46" s="1" t="s">
         <v>227</v>
       </c>
-      <c r="C46" s="1" t="s">
+      <c r="D46" s="1" t="s">
+        <v>226</v>
+      </c>
+      <c r="E46" s="1" t="s">
         <v>228</v>
       </c>
-      <c r="D46" s="1" t="s">
-        <v>229</v>
-      </c>
-      <c r="E46" s="1" t="s">
-        <v>230</v>
-      </c>
       <c r="F46" s="1" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H46" s="1" t="n">
         <v>1</v>
@@ -2278,34 +2256,8 @@
         <v>17</v>
       </c>
     </row>
-    <row r="47" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="1" t="s">
-        <v>231</v>
-      </c>
-      <c r="B47" s="1" t="s">
-        <v>232</v>
-      </c>
-      <c r="C47" s="1" t="s">
-        <v>233</v>
-      </c>
-      <c r="D47" s="1" t="s">
-        <v>232</v>
-      </c>
-      <c r="E47" s="1" t="s">
-        <v>234</v>
-      </c>
-      <c r="F47" s="1" t="n">
-        <v>2</v>
-      </c>
-      <c r="H47" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="L47" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:L47"/>
+  <autoFilter ref="A1:L46"/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.025" bottom="1.025" header="0.7875" footer="0.7875"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" firstPageNumber="1" useFirstPageNumber="true" horizontalDpi="300" verticalDpi="300" copies="1"/>

</xml_diff>

<commit_message>
Fixed U1 (see Build notes 260410), updated BOMs
</commit_message>
<xml_diff>
--- a/kicad/production/DCDCv9-3_Mouser_BOM_for_PCBA.xlsx
+++ b/kicad/production/DCDCv9-3_Mouser_BOM_for_PCBA.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="316" uniqueCount="229">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="315" uniqueCount="228">
   <si>
     <t xml:space="preserve">Reference</t>
   </si>
@@ -628,16 +628,13 @@
     <t xml:space="preserve">U1</t>
   </si>
   <si>
-    <t xml:space="preserve">TBA 1-1212HI</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.mouser.de/ProductDetail/TRACO-Power/TBA-1-1212HI?qs=byeeYqUIh0N5pnK9BA%252B2og%3D%3D</t>
+    <t xml:space="preserve">RP-1212S</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.mouser.de/ProductDetail/RECOM-Power/RP-1212S?qs=YWgezujkI1KjTZkjNYMtQA%3D%3D</t>
   </si>
   <si>
     <t xml:space="preserve">DCDC-Footprints:Converter_DCDC_TRACO_TBA 1-1212HI-3kV-iso</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PEME1-S12-S12-S has lower current consumption but is out of stock</t>
   </si>
   <si>
     <t xml:space="preserve">U12</t>
@@ -790,15 +787,15 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -952,6 +949,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="97.42"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="149.45"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="7.27"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="13" style="1" width="11.53"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1352,10 +1350,10 @@
       <c r="B15" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="C15" s="0" t="s">
+      <c r="C15" s="1" t="s">
         <v>82</v>
       </c>
-      <c r="D15" s="3" t="s">
+      <c r="D15" s="2" t="s">
         <v>83</v>
       </c>
       <c r="E15" s="2" t="s">
@@ -1381,10 +1379,10 @@
       <c r="B16" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="C16" s="0" t="s">
+      <c r="C16" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="D16" s="3" t="s">
+      <c r="D16" s="2" t="s">
         <v>88</v>
       </c>
       <c r="E16" s="2" t="s">
@@ -2107,11 +2105,9 @@
       <c r="F41" s="1" t="n">
         <v>1</v>
       </c>
+      <c r="G41" s="3"/>
       <c r="H41" s="1" t="n">
         <v>1</v>
-      </c>
-      <c r="J41" s="1" t="s">
-        <v>204</v>
       </c>
       <c r="L41" s="1" t="s">
         <v>17</v>
@@ -2119,28 +2115,28 @@
     </row>
     <row r="42" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="1" t="s">
+        <v>204</v>
+      </c>
+      <c r="B42" s="1" t="s">
         <v>205</v>
       </c>
-      <c r="B42" s="1" t="s">
+      <c r="C42" s="1" t="s">
         <v>206</v>
       </c>
-      <c r="C42" s="1" t="s">
+      <c r="D42" s="1" t="s">
         <v>207</v>
       </c>
-      <c r="D42" s="1" t="s">
+      <c r="E42" s="1" t="s">
         <v>208</v>
       </c>
-      <c r="E42" s="1" t="s">
+      <c r="F42" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="I42" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="K42" s="1" t="s">
         <v>209</v>
-      </c>
-      <c r="F42" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="I42" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="K42" s="1" t="s">
-        <v>210</v>
       </c>
       <c r="L42" s="1" t="s">
         <v>17</v>
@@ -2148,28 +2144,28 @@
     </row>
     <row r="43" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="1" t="s">
+        <v>210</v>
+      </c>
+      <c r="B43" s="1" t="s">
         <v>211</v>
       </c>
-      <c r="B43" s="1" t="s">
+      <c r="C43" s="1" t="s">
         <v>212</v>
       </c>
-      <c r="C43" s="1" t="s">
+      <c r="D43" s="1" t="s">
+        <v>211</v>
+      </c>
+      <c r="E43" s="1" t="s">
         <v>213</v>
       </c>
-      <c r="D43" s="1" t="s">
-        <v>212</v>
-      </c>
-      <c r="E43" s="1" t="s">
+      <c r="F43" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="H43" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="K43" s="1" t="s">
         <v>214</v>
-      </c>
-      <c r="F43" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="H43" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="K43" s="1" t="s">
-        <v>215</v>
       </c>
       <c r="L43" s="1" t="s">
         <v>17</v>
@@ -2177,28 +2173,28 @@
     </row>
     <row r="44" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="1" t="s">
+        <v>215</v>
+      </c>
+      <c r="B44" s="1" t="s">
         <v>216</v>
       </c>
-      <c r="B44" s="1" t="s">
+      <c r="C44" s="1" t="s">
         <v>217</v>
       </c>
-      <c r="C44" s="1" t="s">
+      <c r="D44" s="1" t="s">
+        <v>216</v>
+      </c>
+      <c r="E44" s="1" t="s">
+        <v>213</v>
+      </c>
+      <c r="F44" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="H44" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="J44" s="1" t="s">
         <v>218</v>
-      </c>
-      <c r="D44" s="1" t="s">
-        <v>217</v>
-      </c>
-      <c r="E44" s="1" t="s">
-        <v>214</v>
-      </c>
-      <c r="F44" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="H44" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="J44" s="1" t="s">
-        <v>219</v>
       </c>
       <c r="L44" s="1" t="s">
         <v>17</v>
@@ -2206,19 +2202,19 @@
     </row>
     <row r="45" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="1" t="s">
+        <v>219</v>
+      </c>
+      <c r="B45" s="1" t="s">
         <v>220</v>
       </c>
-      <c r="B45" s="1" t="s">
+      <c r="C45" s="1" t="s">
         <v>221</v>
       </c>
-      <c r="C45" s="1" t="s">
+      <c r="D45" s="1" t="s">
         <v>222</v>
       </c>
-      <c r="D45" s="1" t="s">
+      <c r="E45" s="1" t="s">
         <v>223</v>
-      </c>
-      <c r="E45" s="1" t="s">
-        <v>224</v>
       </c>
       <c r="F45" s="1" t="n">
         <v>1</v>
@@ -2232,19 +2228,19 @@
     </row>
     <row r="46" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="1" t="s">
+        <v>224</v>
+      </c>
+      <c r="B46" s="1" t="s">
         <v>225</v>
       </c>
-      <c r="B46" s="1" t="s">
+      <c r="C46" s="1" t="s">
         <v>226</v>
       </c>
-      <c r="C46" s="1" t="s">
+      <c r="D46" s="1" t="s">
+        <v>225</v>
+      </c>
+      <c r="E46" s="1" t="s">
         <v>227</v>
-      </c>
-      <c r="D46" s="1" t="s">
-        <v>226</v>
-      </c>
-      <c r="E46" s="1" t="s">
-        <v>228</v>
       </c>
       <c r="F46" s="1" t="n">
         <v>2</v>

</xml_diff>